<commit_message>
Fixed leap year issues.
Signed-off-by: lorenzozapparoli <164523426+lorenzozapparoli@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/HP/HP_input/configuration_files/RLC_parameters.xlsx
+++ b/HP/HP_input/configuration_files/RLC_parameters.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\14914\Desktop\lectures\SwissPDGs-TimeSeries\HP\configuration_files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lzapparoli\PycharmProjects\SwissPDGs-TimeSeries\HP\HP_input\configuration_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{312FB3D9-2A4E-439B-A8D7-3B72AD1247FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51C7704B-892F-491F-8587-CE511B1E01E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" tabRatio="693" activeTab="2" xr2:uid="{4E3571C4-5A43-4FA7-B5E7-AC189FF9742A}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" tabRatio="693" activeTab="4" xr2:uid="{4E3571C4-5A43-4FA7-B5E7-AC189FF9742A}"/>
   </bookViews>
   <sheets>
     <sheet name="Multi_Family_House" sheetId="1" r:id="rId1"/>
@@ -197,7 +197,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color theme="1"/>
@@ -686,50 +686,50 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="41"/>
   </cellXfs>
   <cellStyles count="44">
-    <cellStyle name="20% - 着色 1" xfId="18" builtinId="30" customBuiltin="1"/>
-    <cellStyle name="20% - 着色 2" xfId="22" builtinId="34" customBuiltin="1"/>
-    <cellStyle name="20% - 着色 3" xfId="26" builtinId="38" customBuiltin="1"/>
-    <cellStyle name="20% - 着色 4" xfId="30" builtinId="42" customBuiltin="1"/>
-    <cellStyle name="20% - 着色 5" xfId="34" builtinId="46" customBuiltin="1"/>
-    <cellStyle name="20% - 着色 6" xfId="38" builtinId="50" customBuiltin="1"/>
-    <cellStyle name="40% - 着色 1" xfId="19" builtinId="31" customBuiltin="1"/>
-    <cellStyle name="40% - 着色 2" xfId="23" builtinId="35" customBuiltin="1"/>
-    <cellStyle name="40% - 着色 3" xfId="27" builtinId="39" customBuiltin="1"/>
-    <cellStyle name="40% - 着色 4" xfId="31" builtinId="43" customBuiltin="1"/>
-    <cellStyle name="40% - 着色 5" xfId="35" builtinId="47" customBuiltin="1"/>
-    <cellStyle name="40% - 着色 6" xfId="39" builtinId="51" customBuiltin="1"/>
-    <cellStyle name="60% - 着色 1" xfId="20" builtinId="32" customBuiltin="1"/>
-    <cellStyle name="60% - 着色 2" xfId="24" builtinId="36" customBuiltin="1"/>
-    <cellStyle name="60% - 着色 3" xfId="28" builtinId="40" customBuiltin="1"/>
-    <cellStyle name="60% - 着色 4" xfId="32" builtinId="44" customBuiltin="1"/>
-    <cellStyle name="60% - 着色 5" xfId="36" builtinId="48" customBuiltin="1"/>
-    <cellStyle name="60% - 着色 6" xfId="40" builtinId="52" customBuiltin="1"/>
+    <cellStyle name="20% - Accent1" xfId="18" builtinId="30" customBuiltin="1"/>
+    <cellStyle name="20% - Accent2" xfId="22" builtinId="34" customBuiltin="1"/>
+    <cellStyle name="20% - Accent3" xfId="26" builtinId="38" customBuiltin="1"/>
+    <cellStyle name="20% - Accent4" xfId="30" builtinId="42" customBuiltin="1"/>
+    <cellStyle name="20% - Accent5" xfId="34" builtinId="46" customBuiltin="1"/>
+    <cellStyle name="20% - Accent6" xfId="38" builtinId="50" customBuiltin="1"/>
+    <cellStyle name="40% - Accent1" xfId="19" builtinId="31" customBuiltin="1"/>
+    <cellStyle name="40% - Accent2" xfId="23" builtinId="35" customBuiltin="1"/>
+    <cellStyle name="40% - Accent3" xfId="27" builtinId="39" customBuiltin="1"/>
+    <cellStyle name="40% - Accent4" xfId="31" builtinId="43" customBuiltin="1"/>
+    <cellStyle name="40% - Accent5" xfId="35" builtinId="47" customBuiltin="1"/>
+    <cellStyle name="40% - Accent6" xfId="39" builtinId="51" customBuiltin="1"/>
+    <cellStyle name="60% - Accent1" xfId="20" builtinId="32" customBuiltin="1"/>
+    <cellStyle name="60% - Accent2" xfId="24" builtinId="36" customBuiltin="1"/>
+    <cellStyle name="60% - Accent3" xfId="28" builtinId="40" customBuiltin="1"/>
+    <cellStyle name="60% - Accent4" xfId="32" builtinId="44" customBuiltin="1"/>
+    <cellStyle name="60% - Accent5" xfId="36" builtinId="48" customBuiltin="1"/>
+    <cellStyle name="60% - Accent6" xfId="40" builtinId="52" customBuiltin="1"/>
+    <cellStyle name="Accent1" xfId="17" builtinId="29" customBuiltin="1"/>
+    <cellStyle name="Accent2" xfId="21" builtinId="33" customBuiltin="1"/>
+    <cellStyle name="Accent3" xfId="25" builtinId="37" customBuiltin="1"/>
+    <cellStyle name="Accent4" xfId="29" builtinId="41" customBuiltin="1"/>
+    <cellStyle name="Accent5" xfId="33" builtinId="45" customBuiltin="1"/>
+    <cellStyle name="Accent6" xfId="37" builtinId="49" customBuiltin="1"/>
+    <cellStyle name="Bad" xfId="7" builtinId="27" customBuiltin="1"/>
+    <cellStyle name="Calculation" xfId="11" builtinId="22" customBuiltin="1"/>
+    <cellStyle name="Check Cell" xfId="13" builtinId="23" customBuiltin="1"/>
+    <cellStyle name="Explanatory Text" xfId="15" builtinId="53" customBuiltin="1"/>
+    <cellStyle name="Good" xfId="6" builtinId="26" customBuiltin="1"/>
+    <cellStyle name="Heading 1" xfId="2" builtinId="16" customBuiltin="1"/>
+    <cellStyle name="Heading 2" xfId="3" builtinId="17" customBuiltin="1"/>
+    <cellStyle name="Heading 3" xfId="4" builtinId="18" customBuiltin="1"/>
+    <cellStyle name="Heading 4" xfId="5" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="Input" xfId="9" builtinId="20" customBuiltin="1"/>
+    <cellStyle name="Linked Cell" xfId="12" builtinId="24" customBuiltin="1"/>
+    <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="41" xr:uid="{4ECC4F70-F5C6-47DB-A59F-AB35C131844A}"/>
     <cellStyle name="Note 2" xfId="43" xr:uid="{475F5818-A1C8-4D71-84F8-0BA94BD8DF32}"/>
+    <cellStyle name="Output" xfId="10" builtinId="21" customBuiltin="1"/>
     <cellStyle name="Percent 2" xfId="42" xr:uid="{2828ECCD-A316-4C9A-A7B8-5EF1D4BA8D3E}"/>
-    <cellStyle name="标题" xfId="1" builtinId="15" customBuiltin="1"/>
-    <cellStyle name="标题 1" xfId="2" builtinId="16" customBuiltin="1"/>
-    <cellStyle name="标题 2" xfId="3" builtinId="17" customBuiltin="1"/>
-    <cellStyle name="标题 3" xfId="4" builtinId="18" customBuiltin="1"/>
-    <cellStyle name="标题 4" xfId="5" builtinId="19" customBuiltin="1"/>
-    <cellStyle name="差" xfId="7" builtinId="27" customBuiltin="1"/>
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="好" xfId="6" builtinId="26" customBuiltin="1"/>
-    <cellStyle name="汇总" xfId="16" builtinId="25" customBuiltin="1"/>
-    <cellStyle name="计算" xfId="11" builtinId="22" customBuiltin="1"/>
-    <cellStyle name="检查单元格" xfId="13" builtinId="23" customBuiltin="1"/>
-    <cellStyle name="解释性文本" xfId="15" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="警告文本" xfId="14" builtinId="11" customBuiltin="1"/>
-    <cellStyle name="链接单元格" xfId="12" builtinId="24" customBuiltin="1"/>
-    <cellStyle name="适中" xfId="8" builtinId="28" customBuiltin="1"/>
-    <cellStyle name="输出" xfId="10" builtinId="21" customBuiltin="1"/>
-    <cellStyle name="输入" xfId="9" builtinId="20" customBuiltin="1"/>
-    <cellStyle name="着色 1" xfId="17" builtinId="29" customBuiltin="1"/>
-    <cellStyle name="着色 2" xfId="21" builtinId="33" customBuiltin="1"/>
-    <cellStyle name="着色 3" xfId="25" builtinId="37" customBuiltin="1"/>
-    <cellStyle name="着色 4" xfId="29" builtinId="41" customBuiltin="1"/>
-    <cellStyle name="着色 5" xfId="33" builtinId="45" customBuiltin="1"/>
-    <cellStyle name="着色 6" xfId="37" builtinId="49" customBuiltin="1"/>
+    <cellStyle name="Title" xfId="1" builtinId="15" customBuiltin="1"/>
+    <cellStyle name="Total" xfId="16" builtinId="25" customBuiltin="1"/>
+    <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -781,7 +781,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 主题">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
     <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
@@ -1078,14 +1078,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4887061F-8787-43BE-B6A9-0F015D108F3A}">
   <dimension ref="A1:J10"/>
-  <sheetFormatPr defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.9296875" customWidth="1"/>
-    <col min="2" max="2" width="19.59765625" customWidth="1"/>
-    <col min="3" max="4" width="9.46484375" customWidth="1"/>
+    <col min="1" max="1" width="13.90625" customWidth="1"/>
+    <col min="2" max="2" width="19.6328125" customWidth="1"/>
+    <col min="3" max="4" width="9.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
         <v>13</v>
       </c>
@@ -1111,7 +1111,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -1143,7 +1143,7 @@
         <v>2605</v>
       </c>
     </row>
-    <row r="3" spans="1:10">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -1175,7 +1175,7 @@
         <v>1554</v>
       </c>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>1</v>
       </c>
@@ -1207,7 +1207,7 @@
         <v>2164</v>
       </c>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -1239,7 +1239,7 @@
         <v>3040</v>
       </c>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -1271,7 +1271,7 @@
         <v>3175</v>
       </c>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -1303,7 +1303,7 @@
         <v>2613</v>
       </c>
     </row>
-    <row r="8" spans="1:10">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -1335,7 +1335,7 @@
         <v>1447</v>
       </c>
     </row>
-    <row r="9" spans="1:10">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>5</v>
       </c>
@@ -1367,7 +1367,7 @@
         <v>1359</v>
       </c>
     </row>
-    <row r="10" spans="1:10">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>6</v>
       </c>
@@ -1412,13 +1412,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66B55B15-1B91-49C2-AB9F-CCC86673EA28}">
   <dimension ref="A1:J10"/>
-  <sheetFormatPr defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.9296875" customWidth="1"/>
-    <col min="2" max="4" width="9.46484375" customWidth="1"/>
+    <col min="1" max="1" width="13.90625" customWidth="1"/>
+    <col min="2" max="4" width="9.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
         <v>13</v>
       </c>
@@ -1444,7 +1444,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -1476,7 +1476,7 @@
         <v>2884</v>
       </c>
     </row>
-    <row r="3" spans="1:10">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -1508,7 +1508,7 @@
         <v>2568</v>
       </c>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>1</v>
       </c>
@@ -1540,7 +1540,7 @@
         <v>3359</v>
       </c>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -1572,7 +1572,7 @@
         <v>3334</v>
       </c>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -1604,7 +1604,7 @@
         <v>4344</v>
       </c>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -1636,7 +1636,7 @@
         <v>4259</v>
       </c>
     </row>
-    <row r="8" spans="1:10">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -1668,7 +1668,7 @@
         <v>2204</v>
       </c>
     </row>
-    <row r="9" spans="1:10">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>5</v>
       </c>
@@ -1700,7 +1700,7 @@
         <v>1536</v>
       </c>
     </row>
-    <row r="10" spans="1:10">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>6</v>
       </c>
@@ -1745,12 +1745,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40DFEC1B-336B-4B02-964B-F1CF6053B8EE}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.46484375" customWidth="1"/>
+    <col min="1" max="1" width="19.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>28</v>
       </c>
@@ -1758,7 +1758,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -1766,7 +1766,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -1774,7 +1774,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1792,14 +1792,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BD1514E-A0C2-4A4B-AC42-0DB308F55B41}">
   <dimension ref="A1:F5"/>
-  <sheetFormatPr defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="13.19921875" customWidth="1"/>
-    <col min="3" max="3" width="19.33203125" customWidth="1"/>
-    <col min="4" max="4" width="18.59765625" customWidth="1"/>
+    <col min="2" max="2" width="13.1796875" customWidth="1"/>
+    <col min="3" max="3" width="19.36328125" customWidth="1"/>
+    <col min="4" max="4" width="18.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>13</v>
       </c>
@@ -1819,7 +1819,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>0</v>
       </c>
@@ -1839,7 +1839,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1980</v>
       </c>
@@ -1859,7 +1859,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2000</v>
       </c>
@@ -1879,7 +1879,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2010</v>
       </c>
@@ -1909,12 +1909,12 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F4910E2-C354-42F7-99A7-C44CBCE9E6A2}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.19921875" customWidth="1"/>
+    <col min="1" max="1" width="11.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>22</v>
       </c>
@@ -1925,7 +1925,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -1936,7 +1936,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -1947,7 +1947,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1958,7 +1958,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>21</v>
       </c>
@@ -1979,9 +1979,9 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{935D386D-459F-4703-98C6-470C782C9C4E}">
   <dimension ref="A1:H35"/>
-  <sheetFormatPr defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
         <v>29</v>
       </c>
@@ -1995,7 +1995,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="14.25">
+    <row r="2" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -2015,7 +2015,7 @@
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
     </row>
-    <row r="3" spans="1:8" ht="14.25">
+    <row r="3" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -2035,7 +2035,7 @@
       <c r="G3" s="1"/>
       <c r="H3" s="1"/>
     </row>
-    <row r="4" spans="1:8">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>1</v>
       </c>
@@ -2052,7 +2052,7 @@
         <v>2.5497851575737034</v>
       </c>
     </row>
-    <row r="5" spans="1:8">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -2069,7 +2069,7 @@
         <v>2.5624547879260988</v>
       </c>
     </row>
-    <row r="6" spans="1:8">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -2086,7 +2086,7 @@
         <v>2.1617623263282275</v>
       </c>
     </row>
-    <row r="7" spans="1:8">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -2103,7 +2103,7 @@
         <v>1.41558347107438</v>
       </c>
     </row>
-    <row r="8" spans="1:8">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -2120,7 +2120,7 @@
         <v>1.1838696971327518</v>
       </c>
     </row>
-    <row r="9" spans="1:8">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>5</v>
       </c>
@@ -2137,7 +2137,7 @@
         <v>0.93913392857142852</v>
       </c>
     </row>
-    <row r="10" spans="1:8">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>6</v>
       </c>
@@ -2154,18 +2154,18 @@
         <v>0.67253941167315112</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="14.25">
+    <row r="13" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
     </row>
-    <row r="24" spans="3:5" ht="14.25">
+    <row r="24" spans="3:5" ht="14.5" x14ac:dyDescent="0.35">
       <c r="C24" s="1"/>
       <c r="D24" s="1"/>
       <c r="E24" s="1"/>
     </row>
-    <row r="35" spans="3:5" ht="14.25">
+    <row r="35" spans="3:5" ht="14.5" x14ac:dyDescent="0.35">
       <c r="C35" s="1"/>
       <c r="D35" s="1"/>
       <c r="E35" s="1"/>
@@ -2178,9 +2178,9 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{07FF9675-FE0E-4B1F-944B-B707DAF591D5}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
         <v>29</v>
       </c>
@@ -2194,7 +2194,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="14.25">
+    <row r="2" spans="1:5" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -2211,7 +2211,7 @@
         <v>1.7471475834292289</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -2228,7 +2228,7 @@
         <v>2.3478544923807623</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>1</v>
       </c>
@@ -2245,7 +2245,7 @@
         <v>1.6764761480160499</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -2262,7 +2262,7 @@
         <v>1.4971208516953856</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -2279,7 +2279,7 @@
         <v>1.3929935198947572</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -2296,7 +2296,7 @@
         <v>1.06484379972416</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -2313,7 +2313,7 @@
         <v>0.90046584668931084</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>5</v>
       </c>
@@ -2330,7 +2330,7 @@
         <v>0.63121381636136287</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>6</v>
       </c>
@@ -2355,17 +2355,17 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7238586D-2BBF-4871-B563-532B40ED7A98}">
   <dimension ref="A1:Q35"/>
-  <sheetFormatPr defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="11.6640625" customWidth="1"/>
+    <col min="2" max="2" width="11.6328125" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="11.796875" customWidth="1"/>
-    <col min="15" max="15" width="11.796875" customWidth="1"/>
-    <col min="16" max="16" width="19.9296875" customWidth="1"/>
-    <col min="17" max="17" width="17.06640625" customWidth="1"/>
+    <col min="6" max="6" width="11.81640625" customWidth="1"/>
+    <col min="15" max="15" width="11.81640625" customWidth="1"/>
+    <col min="16" max="16" width="19.90625" customWidth="1"/>
+    <col min="17" max="17" width="17.08984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
         <v>29</v>
       </c>
@@ -2412,7 +2412,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="2" spans="1:17" ht="14.25">
+    <row r="2" spans="1:17" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -2464,7 +2464,7 @@
         <v>1.433019026071966</v>
       </c>
     </row>
-    <row r="3" spans="1:17">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -2516,7 +2516,7 @@
         <v>1.7276923076923079</v>
       </c>
     </row>
-    <row r="4" spans="1:17">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>1</v>
       </c>
@@ -2568,7 +2568,7 @@
         <v>1.3782900448164479</v>
       </c>
     </row>
-    <row r="5" spans="1:17">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -2620,7 +2620,7 @@
         <v>1.1038482474226798</v>
       </c>
     </row>
-    <row r="6" spans="1:17">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -2672,7 +2672,7 @@
         <v>1.046276077141659</v>
       </c>
     </row>
-    <row r="7" spans="1:17">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -2689,7 +2689,7 @@
         <v>0.88579901960784324</v>
       </c>
     </row>
-    <row r="8" spans="1:17">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -2706,7 +2706,7 @@
         <v>0.79633860153256697</v>
       </c>
     </row>
-    <row r="9" spans="1:17">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>5</v>
       </c>
@@ -2723,7 +2723,7 @@
         <v>0.59134745380802167</v>
       </c>
     </row>
-    <row r="10" spans="1:17">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>6</v>
       </c>
@@ -2775,14 +2775,14 @@
         <v>0.39614913008347785</v>
       </c>
     </row>
-    <row r="13" spans="1:17" ht="14.25">
+    <row r="13" spans="1:17" ht="14.5" x14ac:dyDescent="0.35">
       <c r="B13" s="1"/>
       <c r="P13" s="1"/>
     </row>
-    <row r="24" spans="16:16" ht="14.25">
+    <row r="24" spans="16:16" ht="14.5" x14ac:dyDescent="0.35">
       <c r="P24" s="1"/>
     </row>
-    <row r="35" spans="16:16" ht="14.25">
+    <row r="35" spans="16:16" ht="14.5" x14ac:dyDescent="0.35">
       <c r="P35" s="1"/>
     </row>
   </sheetData>

</xml_diff>